<commit_message>
added io list filler
</commit_message>
<xml_diff>
--- a/Pipeline2App/assets/ButtonsLayout.xlsx
+++ b/Pipeline2App/assets/ButtonsLayout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Source\Repos\_Openn2\Pipeline2App\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3009E999-4A53-4F52-8A9D-8709B35F1702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2905C541-F3C2-4242-B3F2-1CA0FA88CD8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17790" xr2:uid="{9D6DAE04-F57E-45A2-8B00-3B5708FB93E1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="48">
   <si>
     <t>&gt;</t>
   </si>
@@ -182,6 +182,45 @@
   <si>
     <t>Open
 Empty Shells .xlsm</t>
+  </si>
+  <si>
+    <t>Open
+IO Tags</t>
+  </si>
+  <si>
+    <t>Open
+Data Blocks Folder</t>
+  </si>
+  <si>
+    <t>Open
+Diag Data Folder</t>
+  </si>
+  <si>
+    <t>Open
+Harware Data Folder</t>
+  </si>
+  <si>
+    <t>Open
+I/O List</t>
+  </si>
+  <si>
+    <t>Open
+Cause&amp;Effect Matrix</t>
+  </si>
+  <si>
+    <t>Open
+Fill Config .csv</t>
+  </si>
+  <si>
+    <t>Open
+Signal Types .csv</t>
+  </si>
+  <si>
+    <t>Open
+Diag Config .csv Folder</t>
+  </si>
+  <si>
+    <t>Validation Logs Folder</t>
   </si>
 </sst>
 </file>
@@ -678,287 +717,297 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45AF97D9-B137-4003-B959-FBB2624648E9}">
-  <dimension ref="A2:S27"/>
+  <dimension ref="B2:T30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.28515625" customWidth="1"/>
-    <col min="3" max="3" width="20.28515625" customWidth="1"/>
-    <col min="4" max="4" width="5" customWidth="1"/>
-    <col min="5" max="5" width="20.28515625" customWidth="1"/>
-    <col min="6" max="6" width="5" customWidth="1"/>
-    <col min="7" max="7" width="20.28515625" customWidth="1"/>
-    <col min="8" max="8" width="5" customWidth="1"/>
-    <col min="9" max="9" width="20.28515625" customWidth="1"/>
-    <col min="10" max="10" width="5" customWidth="1"/>
-    <col min="11" max="11" width="20.28515625" customWidth="1"/>
-    <col min="12" max="12" width="5" customWidth="1"/>
-    <col min="13" max="13" width="20.28515625" customWidth="1"/>
-    <col min="14" max="14" width="5" customWidth="1"/>
-    <col min="15" max="15" width="20.28515625" customWidth="1"/>
-    <col min="16" max="16" width="5" customWidth="1"/>
-    <col min="17" max="17" width="20.28515625" customWidth="1"/>
-    <col min="18" max="18" width="5" customWidth="1"/>
-    <col min="19" max="19" width="20.28515625" customWidth="1"/>
+    <col min="1" max="1" width="5.140625" customWidth="1"/>
+    <col min="2" max="2" width="20.28515625" customWidth="1"/>
+    <col min="4" max="4" width="20.28515625" customWidth="1"/>
+    <col min="5" max="5" width="5" customWidth="1"/>
+    <col min="6" max="6" width="20.28515625" customWidth="1"/>
+    <col min="7" max="7" width="5" customWidth="1"/>
+    <col min="8" max="8" width="20.28515625" customWidth="1"/>
+    <col min="9" max="9" width="5" customWidth="1"/>
+    <col min="10" max="10" width="20.28515625" customWidth="1"/>
+    <col min="11" max="11" width="5" customWidth="1"/>
+    <col min="12" max="12" width="20.28515625" customWidth="1"/>
+    <col min="13" max="13" width="5" customWidth="1"/>
+    <col min="14" max="14" width="20.28515625" customWidth="1"/>
+    <col min="15" max="15" width="5" customWidth="1"/>
+    <col min="16" max="16" width="20.28515625" customWidth="1"/>
+    <col min="17" max="17" width="5" customWidth="1"/>
+    <col min="18" max="18" width="20.28515625" customWidth="1"/>
+    <col min="19" max="19" width="5" customWidth="1"/>
+    <col min="20" max="20" width="20.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:19" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
+    <row r="2" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:20" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="D3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="F3" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="H3" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="J3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="L3" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="L3" s="4" t="s">
+      <c r="M3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="M3" s="7" t="s">
+      <c r="N3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="O3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="P3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="Q3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="Q3" s="7" t="s">
+      <c r="R3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="R3" s="4" t="s">
+      <c r="S3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="S3" s="7" t="s">
+      <c r="T3" s="7" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="C4" s="5" t="s">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="D4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="H4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="J4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="L4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="M4" s="5" t="s">
+      <c r="N4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="O4" s="5" t="s">
+      <c r="P4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="Q4" s="5" t="s">
+      <c r="R4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="S4" s="5" t="s">
+      <c r="T4" s="5" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="60" x14ac:dyDescent="0.25">
-      <c r="A5" s="6"/>
+    <row r="5" spans="2:20" ht="60" x14ac:dyDescent="0.25">
       <c r="B5" s="6"/>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="6"/>
+      <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="6"/>
+      <c r="F5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="6"/>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="6"/>
+      <c r="H5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H5" s="6"/>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="6"/>
+      <c r="J5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J5" s="6"/>
-      <c r="K5" s="3" t="s">
+      <c r="K5" s="6"/>
+      <c r="L5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="6"/>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="6"/>
+      <c r="N5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="N5" s="6"/>
-      <c r="O5" s="3" t="s">
+      <c r="O5" s="6"/>
+      <c r="P5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="P5" s="6"/>
-      <c r="Q5" s="3" t="s">
+      <c r="Q5" s="6"/>
+      <c r="R5" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="R5" s="6"/>
-      <c r="S5" s="3" t="s">
+      <c r="S5" s="6"/>
+      <c r="T5" s="3" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A6" s="6"/>
+    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B6" s="6"/>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="6"/>
+      <c r="D6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="2" t="s">
+      <c r="E6" s="6"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="H6" s="6"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="2" t="s">
+      <c r="I6" s="6"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="L6" s="6"/>
-      <c r="M6" s="2" t="s">
+      <c r="M6" s="6"/>
+      <c r="N6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="N6" s="6"/>
-      <c r="O6" s="2" t="s">
+      <c r="O6" s="6"/>
+      <c r="P6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="2" t="s">
+      <c r="Q6" s="6"/>
+      <c r="R6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="R6" s="6"/>
-      <c r="S6" s="2"/>
-    </row>
-    <row r="7" spans="1:19" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6"/>
+      <c r="S6" s="6"/>
+      <c r="T6" s="2"/>
+    </row>
+    <row r="7" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="6"/>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="6"/>
+      <c r="D7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="6"/>
       <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="3" t="s">
+      <c r="F7" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" s="6"/>
+      <c r="H7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="H7" s="6"/>
-      <c r="I7" s="8" t="s">
+      <c r="I7" s="6"/>
+      <c r="J7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="J7" s="6"/>
-      <c r="K7" s="3" t="s">
+      <c r="K7" s="6"/>
+      <c r="L7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="L7" s="6"/>
-      <c r="M7" s="3" t="s">
+      <c r="M7" s="6"/>
+      <c r="N7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="N7" s="6"/>
-      <c r="O7" s="3" t="s">
+      <c r="O7" s="6"/>
+      <c r="P7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="3" t="s">
+      <c r="Q7" s="6"/>
+      <c r="R7" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="R7" s="6"/>
-      <c r="S7" s="3" t="s">
+      <c r="S7" s="6"/>
+      <c r="T7" s="3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A8" s="6"/>
+    <row r="8" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B8" s="6"/>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="6"/>
+      <c r="D8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="6"/>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="2" t="s">
+      <c r="G8" s="6"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="6"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="6"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="6"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="6"/>
+      <c r="R8" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="R8" s="6"/>
-      <c r="S8" s="2"/>
-    </row>
-    <row r="9" spans="1:19" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
+      <c r="S8" s="6"/>
+      <c r="T8" s="2"/>
+    </row>
+    <row r="9" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="6"/>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="6"/>
+      <c r="D9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="6"/>
       <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="8" t="s">
+      <c r="F9" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" s="6"/>
+      <c r="H9" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="6"/>
-      <c r="I9" s="9" t="s">
+      <c r="I9" s="6"/>
+      <c r="J9" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="J9" s="6"/>
       <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
+      <c r="L9" s="8" t="s">
+        <v>38</v>
+      </c>
       <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
+      <c r="N9" s="8" t="s">
+        <v>40</v>
+      </c>
       <c r="O9" s="6"/>
-      <c r="P9" s="6"/>
-      <c r="Q9" s="3" t="s">
+      <c r="P9" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q9" s="6"/>
+      <c r="R9" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="R9" s="6"/>
-      <c r="S9" s="8" t="s">
+      <c r="S9" s="6"/>
+      <c r="T9" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A10" s="6"/>
+    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B10" s="6"/>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="6"/>
+      <c r="D10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
@@ -974,308 +1023,319 @@
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
       <c r="S10" s="6"/>
-    </row>
-    <row r="11" spans="1:19" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
+      <c r="T10" s="6"/>
+    </row>
+    <row r="11" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="6"/>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="6"/>
+      <c r="D11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="6"/>
       <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
+      <c r="F11" s="8" t="s">
+        <v>45</v>
+      </c>
       <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="J11" s="6"/>
+      <c r="I11" s="6"/>
       <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
+      <c r="L11" s="8" t="s">
+        <v>39</v>
+      </c>
       <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
+      <c r="N11" s="8" t="s">
+        <v>46</v>
+      </c>
       <c r="O11" s="6"/>
       <c r="P11" s="6"/>
-      <c r="Q11" s="8" t="s">
+      <c r="Q11" s="6"/>
+      <c r="R11" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="R11" s="6"/>
       <c r="S11" s="6"/>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A12" s="6"/>
+      <c r="T11" s="6"/>
+    </row>
+    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B12" s="6"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="6"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="6"/>
-      <c r="S12" s="2"/>
-    </row>
-    <row r="13" spans="1:19" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="6"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="6"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="6"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="6"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="6"/>
+      <c r="T12" s="2"/>
+    </row>
+    <row r="13" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="6"/>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="6"/>
+      <c r="D13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="6"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="6"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="6"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="2"/>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A14" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="6"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="6"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="6"/>
+      <c r="R13" s="2"/>
+      <c r="S13" s="6"/>
+      <c r="T13" s="2"/>
+    </row>
+    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B14" s="6"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="2"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="6"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="6"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="6"/>
-      <c r="S14" s="2"/>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A15" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="2"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="6"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="6"/>
+      <c r="N14" s="2"/>
+      <c r="O14" s="6"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="6"/>
+      <c r="R14" s="2"/>
+      <c r="S14" s="6"/>
+      <c r="T14" s="2"/>
+    </row>
+    <row r="15" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="6"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="2"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="6"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="6"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="6"/>
-      <c r="S15" s="2"/>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A16" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="6"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="6"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="6"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="6"/>
+      <c r="R15" s="2"/>
+      <c r="S15" s="6"/>
+      <c r="T15" s="2"/>
+    </row>
+    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B16" s="6"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="6"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="6"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="6"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="6"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="6"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="6"/>
-      <c r="S16" s="2"/>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A17" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="6"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="6"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="6"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="6"/>
+      <c r="R16" s="2"/>
+      <c r="S16" s="6"/>
+      <c r="T16" s="2"/>
+    </row>
+    <row r="17" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="6"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="2"/>
-      <c r="F17" s="6"/>
-      <c r="G17" s="2"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="6"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="6"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="6"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="6"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="6"/>
-      <c r="S17" s="2"/>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A18" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E17" s="6"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="6"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="6"/>
+      <c r="N17" s="2"/>
+      <c r="O17" s="6"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="6"/>
+      <c r="R17" s="2"/>
+      <c r="S17" s="6"/>
+      <c r="T17" s="2"/>
+    </row>
+    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B18" s="6"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="2"/>
-      <c r="L18" s="6"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="6"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="6"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="6"/>
-      <c r="S18" s="2"/>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A19" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="6"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="6"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="6"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="6"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="6"/>
+      <c r="T18" s="2"/>
+    </row>
+    <row r="19" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="6"/>
-      <c r="C19" s="2"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="2"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="6"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="6"/>
-      <c r="O19" s="2"/>
-      <c r="P19" s="6"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="6"/>
-      <c r="S19" s="2"/>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A20" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E19" s="6"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="6"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="6"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="6"/>
+      <c r="R19" s="2"/>
+      <c r="S19" s="6"/>
+      <c r="T19" s="2"/>
+    </row>
+    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B20" s="6"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="6"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="6"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="6"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="6"/>
-      <c r="O20" s="1"/>
-      <c r="P20" s="6"/>
-      <c r="Q20" s="1"/>
-      <c r="R20" s="6"/>
-      <c r="S20" s="1"/>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A21" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="6"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="6"/>
+      <c r="N20" s="2"/>
+      <c r="O20" s="6"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="6"/>
+      <c r="R20" s="2"/>
+      <c r="S20" s="6"/>
+      <c r="T20" s="2"/>
+    </row>
+    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B21" s="6"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="6"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="6"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="6"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="6"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="6"/>
-      <c r="Q21" s="1"/>
-      <c r="R21" s="6"/>
-      <c r="S21" s="1"/>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A22" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="6"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="6"/>
+      <c r="L21" s="2"/>
+      <c r="M21" s="6"/>
+      <c r="N21" s="2"/>
+      <c r="O21" s="6"/>
+      <c r="P21" s="2"/>
+      <c r="Q21" s="6"/>
+      <c r="R21" s="2"/>
+      <c r="S21" s="6"/>
+      <c r="T21" s="2"/>
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
-      <c r="D22" s="6"/>
+      <c r="D22" s="2"/>
       <c r="E22" s="6"/>
-      <c r="F22" s="6"/>
+      <c r="F22" s="2"/>
       <c r="G22" s="6"/>
-      <c r="H22" s="6"/>
+      <c r="H22" s="2"/>
       <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
+      <c r="J22" s="2"/>
       <c r="K22" s="6"/>
-      <c r="L22" s="6"/>
+      <c r="L22" s="2"/>
       <c r="M22" s="6"/>
-      <c r="N22" s="6"/>
+      <c r="N22" s="2"/>
       <c r="O22" s="6"/>
-      <c r="P22" s="6"/>
+      <c r="P22" s="2"/>
       <c r="Q22" s="6"/>
-      <c r="R22" s="6"/>
+      <c r="R22" s="2"/>
       <c r="S22" s="6"/>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A23" s="6"/>
+      <c r="T22" s="2"/>
+    </row>
+    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
-      <c r="D23" s="6"/>
+      <c r="D23" s="1"/>
       <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
+      <c r="F23" s="1"/>
       <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
+      <c r="H23" s="1"/>
       <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
+      <c r="J23" s="1"/>
       <c r="K23" s="6"/>
-      <c r="L23" s="6"/>
+      <c r="L23" s="1"/>
       <c r="M23" s="6"/>
-      <c r="N23" s="6"/>
+      <c r="N23" s="1"/>
       <c r="O23" s="6"/>
-      <c r="P23" s="6"/>
+      <c r="P23" s="1"/>
       <c r="Q23" s="6"/>
-      <c r="R23" s="6"/>
+      <c r="R23" s="1"/>
       <c r="S23" s="6"/>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A24" s="6"/>
+      <c r="T23" s="1"/>
+    </row>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
+      <c r="D24" s="1"/>
       <c r="E24" s="6"/>
-      <c r="F24" s="6"/>
+      <c r="F24" s="1"/>
       <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
+      <c r="H24" s="1"/>
       <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
+      <c r="J24" s="1"/>
       <c r="K24" s="6"/>
-      <c r="L24" s="6"/>
+      <c r="L24" s="1"/>
       <c r="M24" s="6"/>
-      <c r="N24" s="6"/>
+      <c r="N24" s="1"/>
       <c r="O24" s="6"/>
-      <c r="P24" s="6"/>
+      <c r="P24" s="1"/>
       <c r="Q24" s="6"/>
-      <c r="R24" s="6"/>
+      <c r="R24" s="1"/>
       <c r="S24" s="6"/>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A25" s="6"/>
+      <c r="T24" s="1"/>
+    </row>
+    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
@@ -1294,9 +1354,9 @@
       <c r="Q25" s="6"/>
       <c r="R25" s="6"/>
       <c r="S25" s="6"/>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A26" s="6"/>
+      <c r="T25" s="6"/>
+    </row>
+    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
@@ -1315,9 +1375,9 @@
       <c r="Q26" s="6"/>
       <c r="R26" s="6"/>
       <c r="S26" s="6"/>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A27" s="6"/>
+      <c r="T26" s="6"/>
+    </row>
+    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
@@ -1336,6 +1396,70 @@
       <c r="Q27" s="6"/>
       <c r="R27" s="6"/>
       <c r="S27" s="6"/>
+      <c r="T27" s="6"/>
+    </row>
+    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B28" s="6"/>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
+      <c r="J28" s="6"/>
+      <c r="K28" s="6"/>
+      <c r="L28" s="6"/>
+      <c r="M28" s="6"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="6"/>
+      <c r="P28" s="6"/>
+      <c r="Q28" s="6"/>
+      <c r="R28" s="6"/>
+      <c r="S28" s="6"/>
+      <c r="T28" s="6"/>
+    </row>
+    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B29" s="6"/>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6"/>
+      <c r="J29" s="6"/>
+      <c r="K29" s="6"/>
+      <c r="L29" s="6"/>
+      <c r="M29" s="6"/>
+      <c r="N29" s="6"/>
+      <c r="O29" s="6"/>
+      <c r="P29" s="6"/>
+      <c r="Q29" s="6"/>
+      <c r="R29" s="6"/>
+      <c r="S29" s="6"/>
+      <c r="T29" s="6"/>
+    </row>
+    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="B30" s="6"/>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="6"/>
+      <c r="J30" s="6"/>
+      <c r="K30" s="6"/>
+      <c r="L30" s="6"/>
+      <c r="M30" s="6"/>
+      <c r="N30" s="6"/>
+      <c r="O30" s="6"/>
+      <c r="P30" s="6"/>
+      <c r="Q30" s="6"/>
+      <c r="R30" s="6"/>
+      <c r="S30" s="6"/>
+      <c r="T30" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated documents and parameters
</commit_message>
<xml_diff>
--- a/Pipeline2App/assets/ButtonsLayout.xlsx
+++ b/Pipeline2App/assets/ButtonsLayout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Source\Repos\_Openn2\Pipeline2App\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F70D0DA8-1804-4BDB-A6D1-7C19EC37AF89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAB9BE82-3126-4324-AB66-7E89290DB672}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17790" xr2:uid="{9D6DAE04-F57E-45A2-8B00-3B5708FB93E1}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="55">
   <si>
     <t>&gt;</t>
   </si>
@@ -76,10 +76,6 @@
 IOL-&gt;CEM</t>
   </si>
   <si>
-    <t>Fill
-I/O List</t>
-  </si>
-  <si>
     <t>Stage
 I/O List</t>
   </si>
@@ -108,10 +104,6 @@
 Diag List</t>
   </si>
   <si>
-    <t>Generate
-Diag Blocks</t>
-  </si>
-  <si>
     <t>Interfaces
 Generation</t>
   </si>
@@ -224,6 +216,36 @@
   </si>
   <si>
     <t>Validate Diagnosis Assignments</t>
+  </si>
+  <si>
+    <t>Fill
+IOList Script Type Column</t>
+  </si>
+  <si>
+    <t>Fill
+IOLis Index Column</t>
+  </si>
+  <si>
+    <t>Fill
+IOList Diag Cabinet Column</t>
+  </si>
+  <si>
+    <t>Fill
+IOList Diag Bit Column</t>
+  </si>
+  <si>
+    <t>Generate
+Diag Software Blocks</t>
+  </si>
+  <si>
+    <t>Open
+Generated Blocks Folder</t>
+  </si>
+  <si>
+    <t>Fill Out SWP File</t>
+  </si>
+  <si>
+    <t>Generate SWP File</t>
   </si>
 </sst>
 </file>
@@ -334,7 +356,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -351,7 +373,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -363,6 +384,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -720,10 +747,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45AF97D9-B137-4003-B959-FBB2624648E9}">
-  <dimension ref="B2:T32"/>
+  <dimension ref="A1:T26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.140625" customWidth="1"/>
+    <col min="1" max="1" width="9.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.28515625" customWidth="1"/>
     <col min="4" max="4" width="20.28515625" customWidth="1"/>
     <col min="5" max="5" width="5" customWidth="1"/>
@@ -744,771 +771,491 @@
     <col min="20" max="20" width="20.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:20" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="7" t="s">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D1" s="10">
+        <v>100</v>
+      </c>
+      <c r="F1" s="10">
+        <f>D1+100</f>
+        <v>200</v>
+      </c>
+      <c r="H1" s="10">
+        <f>F1+100</f>
+        <v>300</v>
+      </c>
+      <c r="J1" s="10">
+        <f>H1+100</f>
+        <v>400</v>
+      </c>
+      <c r="L1" s="10">
+        <f>J1+100</f>
+        <v>500</v>
+      </c>
+      <c r="N1" s="10">
+        <f>L1+100</f>
+        <v>600</v>
+      </c>
+      <c r="P1" s="10">
+        <f>N1+100</f>
+        <v>700</v>
+      </c>
+      <c r="R1" s="10">
+        <f>P1+100</f>
+        <v>800</v>
+      </c>
+      <c r="T1" s="10">
+        <f>R1+100</f>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:20" ht="45.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="6" t="s">
         <v>3</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
         <v>2</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="J3" s="7" t="s">
-        <v>18</v>
+      <c r="J3" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="L3" s="6" t="s">
         <v>1</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="N3" s="7" t="s">
-        <v>15</v>
+      <c r="N3" s="6" t="s">
+        <v>14</v>
       </c>
       <c r="O3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="P3" s="7" t="s">
-        <v>19</v>
+      <c r="P3" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="Q3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="R3" s="7" t="s">
-        <v>22</v>
+      <c r="R3" s="6" t="s">
+        <v>20</v>
       </c>
       <c r="S3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="T3" s="7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="2:20" x14ac:dyDescent="0.25">
+      <c r="T3" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="D4" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="P4" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="R4" s="5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="T4" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="2:20" ht="60" x14ac:dyDescent="0.25">
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" ht="60" x14ac:dyDescent="0.25">
+      <c r="A5" s="11">
+        <v>10</v>
+      </c>
       <c r="D5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="6"/>
       <c r="F5" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="6"/>
-      <c r="H5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="I5" s="6"/>
       <c r="J5" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="K5" s="6"/>
-      <c r="L5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="M5" s="6"/>
       <c r="N5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="O5" s="6"/>
+        <v>15</v>
+      </c>
       <c r="P5" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="T5" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" s="2"/>
+      <c r="L6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="T6" s="2"/>
+    </row>
+    <row r="7" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="11">
+        <f>A5+10</f>
         <v>20</v>
       </c>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="S5" s="6"/>
-      <c r="T5" s="3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="I6" s="6"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M6" s="6"/>
-      <c r="N6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="O6" s="6"/>
-      <c r="P6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="S6" s="6"/>
-      <c r="T6" s="2"/>
-    </row>
-    <row r="7" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
       <c r="D7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="6"/>
+      <c r="F7" s="3" t="s">
+        <v>48</v>
+      </c>
       <c r="H7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I7" s="6"/>
-      <c r="J7" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="K7" s="6"/>
+        <v>10</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>32</v>
+      </c>
       <c r="L7" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="M7" s="6"/>
+        <v>13</v>
+      </c>
       <c r="N7" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="O7" s="6"/>
+        <v>51</v>
+      </c>
       <c r="P7" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="R7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="S7" s="6"/>
       <c r="T7" s="3" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="D8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
+        <v>23</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="H8" s="2"/>
-      <c r="I8" s="6"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="6"/>
       <c r="L8" s="2"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="6"/>
+      <c r="N8" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="P8" s="2"/>
-      <c r="Q8" s="6"/>
       <c r="R8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="S8" s="6"/>
+        <v>23</v>
+      </c>
       <c r="T8" s="2"/>
     </row>
-    <row r="9" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
+    <row r="9" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="11">
+        <f>A7+10</f>
+        <v>30</v>
+      </c>
       <c r="D9" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="G9" s="6"/>
-      <c r="H9" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="I9" s="6"/>
-      <c r="J9" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="K9" s="6"/>
-      <c r="L9" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="M9" s="6"/>
-      <c r="N9" s="8" t="s">
+      <c r="F9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="P9" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="R9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="T9" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R10" s="2"/>
+    </row>
+    <row r="11" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="11">
+        <f>A9+10</f>
         <v>40</v>
       </c>
-      <c r="O9" s="6"/>
-      <c r="P9" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="Q9" s="6"/>
-      <c r="R9" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="S9" s="6"/>
-      <c r="T9" s="8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
-      <c r="P10" s="6"/>
-      <c r="Q10" s="6"/>
-      <c r="R10" s="6"/>
-      <c r="S10" s="6"/>
-      <c r="T10" s="6"/>
-    </row>
-    <row r="11" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
       <c r="D11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="R11" s="7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="T12" s="2"/>
+    </row>
+    <row r="13" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="11">
+        <f>A11+10</f>
+        <v>50</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="H13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="N13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="P13" s="2"/>
+      <c r="R13" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="T13" s="2"/>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="P14" s="2"/>
+      <c r="R14" s="2"/>
+      <c r="T14" s="2"/>
+    </row>
+    <row r="15" spans="1:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D15" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="N15" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="P15" s="2"/>
+      <c r="R15" s="2"/>
+      <c r="T15" s="2"/>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="D16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="P16" s="2"/>
+      <c r="R16" s="2"/>
+      <c r="T16" s="2"/>
+    </row>
+    <row r="17" spans="4:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D17" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="H17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="N17" s="2"/>
+      <c r="P17" s="2"/>
+      <c r="R17" s="2"/>
+      <c r="T17" s="2"/>
+    </row>
+    <row r="18" spans="4:20" x14ac:dyDescent="0.25">
+      <c r="D18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="T18" s="2"/>
+    </row>
+    <row r="19" spans="4:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D19" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="N19" s="2"/>
+      <c r="P19" s="2"/>
+      <c r="R19" s="2"/>
+      <c r="T19" s="2"/>
+    </row>
+    <row r="20" spans="4:20" x14ac:dyDescent="0.25">
+      <c r="D20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="N20" s="2"/>
+      <c r="P20" s="2"/>
+      <c r="R20" s="2"/>
+      <c r="T20" s="2"/>
+    </row>
+    <row r="21" spans="4:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="M11" s="6"/>
-      <c r="N11" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="O11" s="6"/>
-      <c r="P11" s="6"/>
-      <c r="Q11" s="6"/>
-      <c r="R11" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="S11" s="6"/>
-      <c r="T11" s="6"/>
-    </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E12" s="6"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="6"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="6"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="6"/>
-      <c r="T12" s="2"/>
-    </row>
-    <row r="13" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E13" s="6"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="6"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="6"/>
-      <c r="T13" s="2"/>
-    </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="2"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="6"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="6"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="6"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="6"/>
-      <c r="T14" s="2"/>
-    </row>
-    <row r="15" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="E15" s="6"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="6"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="6"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="6"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="6"/>
-      <c r="T15" s="2"/>
-    </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="6"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="6"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="6"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="6"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="6"/>
-      <c r="T16" s="2"/>
-    </row>
-    <row r="17" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="E17" s="6"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="6"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="2"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="6"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="6"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="6"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="6"/>
-      <c r="T17" s="2"/>
-    </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B18" s="6"/>
-      <c r="C18" s="6"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="2"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="6"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="6"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="6"/>
-      <c r="R18" s="2"/>
-      <c r="S18" s="6"/>
-      <c r="T18" s="2"/>
-    </row>
-    <row r="19" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="E19" s="6"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="6"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="2"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="6"/>
-      <c r="N19" s="2"/>
-      <c r="O19" s="6"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="6"/>
-      <c r="R19" s="2"/>
-      <c r="S19" s="6"/>
-      <c r="T19" s="2"/>
-    </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="6"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="6"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="6"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="6"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="6"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="6"/>
-      <c r="R20" s="2"/>
-      <c r="S20" s="6"/>
-      <c r="T20" s="2"/>
-    </row>
-    <row r="21" spans="2:20" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E21" s="6"/>
       <c r="F21" s="2"/>
-      <c r="G21" s="6"/>
       <c r="H21" s="2"/>
-      <c r="I21" s="6"/>
       <c r="J21" s="2"/>
-      <c r="K21" s="6"/>
       <c r="L21" s="2"/>
-      <c r="M21" s="6"/>
       <c r="N21" s="2"/>
-      <c r="O21" s="6"/>
       <c r="P21" s="2"/>
-      <c r="Q21" s="6"/>
       <c r="R21" s="2"/>
-      <c r="S21" s="6"/>
       <c r="T21" s="2"/>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B22" s="6"/>
-      <c r="C22" s="6"/>
+    <row r="22" spans="4:20" x14ac:dyDescent="0.25">
       <c r="D22" s="2"/>
-      <c r="E22" s="6"/>
       <c r="F22" s="2"/>
-      <c r="G22" s="6"/>
       <c r="H22" s="2"/>
-      <c r="I22" s="6"/>
       <c r="J22" s="2"/>
-      <c r="K22" s="6"/>
       <c r="L22" s="2"/>
-      <c r="M22" s="6"/>
       <c r="N22" s="2"/>
-      <c r="O22" s="6"/>
       <c r="P22" s="2"/>
-      <c r="Q22" s="6"/>
       <c r="R22" s="2"/>
-      <c r="S22" s="6"/>
       <c r="T22" s="2"/>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B23" s="6"/>
-      <c r="C23" s="6"/>
+    <row r="23" spans="4:20" x14ac:dyDescent="0.25">
       <c r="D23" s="2"/>
-      <c r="E23" s="6"/>
       <c r="F23" s="2"/>
-      <c r="G23" s="6"/>
       <c r="H23" s="2"/>
-      <c r="I23" s="6"/>
       <c r="J23" s="2"/>
-      <c r="K23" s="6"/>
       <c r="L23" s="2"/>
-      <c r="M23" s="6"/>
       <c r="N23" s="2"/>
-      <c r="O23" s="6"/>
       <c r="P23" s="2"/>
-      <c r="Q23" s="6"/>
       <c r="R23" s="2"/>
-      <c r="S23" s="6"/>
       <c r="T23" s="2"/>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
+    <row r="24" spans="4:20" x14ac:dyDescent="0.25">
       <c r="D24" s="2"/>
-      <c r="E24" s="6"/>
       <c r="F24" s="2"/>
-      <c r="G24" s="6"/>
       <c r="H24" s="2"/>
-      <c r="I24" s="6"/>
       <c r="J24" s="2"/>
-      <c r="K24" s="6"/>
       <c r="L24" s="2"/>
-      <c r="M24" s="6"/>
       <c r="N24" s="2"/>
-      <c r="O24" s="6"/>
       <c r="P24" s="2"/>
-      <c r="Q24" s="6"/>
       <c r="R24" s="2"/>
-      <c r="S24" s="6"/>
       <c r="T24" s="2"/>
     </row>
-    <row r="25" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
+    <row r="25" spans="4:20" x14ac:dyDescent="0.25">
       <c r="D25" s="1"/>
-      <c r="E25" s="6"/>
       <c r="F25" s="1"/>
-      <c r="G25" s="6"/>
       <c r="H25" s="1"/>
-      <c r="I25" s="6"/>
       <c r="J25" s="1"/>
-      <c r="K25" s="6"/>
       <c r="L25" s="1"/>
-      <c r="M25" s="6"/>
       <c r="N25" s="1"/>
-      <c r="O25" s="6"/>
       <c r="P25" s="1"/>
-      <c r="Q25" s="6"/>
       <c r="R25" s="1"/>
-      <c r="S25" s="6"/>
       <c r="T25" s="1"/>
     </row>
-    <row r="26" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
+    <row r="26" spans="4:20" x14ac:dyDescent="0.25">
       <c r="D26" s="1"/>
-      <c r="E26" s="6"/>
       <c r="F26" s="1"/>
-      <c r="G26" s="6"/>
       <c r="H26" s="1"/>
-      <c r="I26" s="6"/>
       <c r="J26" s="1"/>
-      <c r="K26" s="6"/>
       <c r="L26" s="1"/>
-      <c r="M26" s="6"/>
       <c r="N26" s="1"/>
-      <c r="O26" s="6"/>
       <c r="P26" s="1"/>
-      <c r="Q26" s="6"/>
       <c r="R26" s="1"/>
-      <c r="S26" s="6"/>
       <c r="T26" s="1"/>
-    </row>
-    <row r="27" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B27" s="6"/>
-      <c r="C27" s="6"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="6"/>
-      <c r="K27" s="6"/>
-      <c r="L27" s="6"/>
-      <c r="M27" s="6"/>
-      <c r="N27" s="6"/>
-      <c r="O27" s="6"/>
-      <c r="P27" s="6"/>
-      <c r="Q27" s="6"/>
-      <c r="R27" s="6"/>
-      <c r="S27" s="6"/>
-      <c r="T27" s="6"/>
-    </row>
-    <row r="28" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B28" s="6"/>
-      <c r="C28" s="6"/>
-      <c r="D28" s="6"/>
-      <c r="E28" s="6"/>
-      <c r="F28" s="6"/>
-      <c r="G28" s="6"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="6"/>
-      <c r="J28" s="6"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="6"/>
-      <c r="M28" s="6"/>
-      <c r="N28" s="6"/>
-      <c r="O28" s="6"/>
-      <c r="P28" s="6"/>
-      <c r="Q28" s="6"/>
-      <c r="R28" s="6"/>
-      <c r="S28" s="6"/>
-      <c r="T28" s="6"/>
-    </row>
-    <row r="29" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B29" s="6"/>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="6"/>
-      <c r="G29" s="6"/>
-      <c r="H29" s="6"/>
-      <c r="I29" s="6"/>
-      <c r="J29" s="6"/>
-      <c r="K29" s="6"/>
-      <c r="L29" s="6"/>
-      <c r="M29" s="6"/>
-      <c r="N29" s="6"/>
-      <c r="O29" s="6"/>
-      <c r="P29" s="6"/>
-      <c r="Q29" s="6"/>
-      <c r="R29" s="6"/>
-      <c r="S29" s="6"/>
-      <c r="T29" s="6"/>
-    </row>
-    <row r="30" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B30" s="6"/>
-      <c r="C30" s="6"/>
-      <c r="D30" s="6"/>
-      <c r="E30" s="6"/>
-      <c r="F30" s="6"/>
-      <c r="G30" s="6"/>
-      <c r="H30" s="6"/>
-      <c r="I30" s="6"/>
-      <c r="J30" s="6"/>
-      <c r="K30" s="6"/>
-      <c r="L30" s="6"/>
-      <c r="M30" s="6"/>
-      <c r="N30" s="6"/>
-      <c r="O30" s="6"/>
-      <c r="P30" s="6"/>
-      <c r="Q30" s="6"/>
-      <c r="R30" s="6"/>
-      <c r="S30" s="6"/>
-      <c r="T30" s="6"/>
-    </row>
-    <row r="31" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B31" s="6"/>
-      <c r="C31" s="6"/>
-      <c r="D31" s="6"/>
-      <c r="E31" s="6"/>
-      <c r="F31" s="6"/>
-      <c r="G31" s="6"/>
-      <c r="H31" s="6"/>
-      <c r="I31" s="6"/>
-      <c r="J31" s="6"/>
-      <c r="K31" s="6"/>
-      <c r="L31" s="6"/>
-      <c r="M31" s="6"/>
-      <c r="N31" s="6"/>
-      <c r="O31" s="6"/>
-      <c r="P31" s="6"/>
-      <c r="Q31" s="6"/>
-      <c r="R31" s="6"/>
-      <c r="S31" s="6"/>
-      <c r="T31" s="6"/>
-    </row>
-    <row r="32" spans="2:20" x14ac:dyDescent="0.25">
-      <c r="B32" s="6"/>
-      <c r="C32" s="6"/>
-      <c r="D32" s="6"/>
-      <c r="E32" s="6"/>
-      <c r="F32" s="6"/>
-      <c r="G32" s="6"/>
-      <c r="H32" s="6"/>
-      <c r="I32" s="6"/>
-      <c r="J32" s="6"/>
-      <c r="K32" s="6"/>
-      <c r="L32" s="6"/>
-      <c r="M32" s="6"/>
-      <c r="N32" s="6"/>
-      <c r="O32" s="6"/>
-      <c r="P32" s="6"/>
-      <c r="Q32" s="6"/>
-      <c r="R32" s="6"/>
-      <c r="S32" s="6"/>
-      <c r="T32" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>